<commit_message>
TICVAI: soft platform waits, next-ready scheduling, Block A dates from one schedule; 12 client questions
- Block A schedule: services start against the platform interfaces from day 3 (kernel,
  idempotency, outbox), reports against seeded data; only their end waits. A person whose next
  ticket is waiting takes the next ready one (as ADAM's board shows). Finish 26 April (10 May
  with hard waits); Block A work ends 10 Nov to 25 Dec; overtime to 2 April 2.2-5.2 h/week
- build-plan-deck takes Block A dates from the schedule (AI engine tasks at their days)
- Development plan, readiness note, ticket text and review workbook regenerated; TICKET-STRUCTURE
  records hard and soft waits
- Decisions Register: 12 new client questions (POS terminal, kitchen display, card terminals,
  NFC/RFID, staff devices, device classes, messaging, accounting, UAE Pass, stores and wallets,
  tourism reporting, named services); client email item 9

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Build Plan.xlsx
+++ b/ticvai/handoff/TICVAI - Build Plan.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>1,991 hours</t>
+          <t>1,268 hours</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1009,11 +1009,11 @@
         <v>1392</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>982</v>
+        <v>1273</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -1051,17 +1051,17 @@
         <v>1392</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1144</v>
+        <v>1352</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, White Label &amp; CMS</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, White Label &amp; CMS, Transport, Food &amp; Beverage, Retail</t>
         </is>
       </c>
     </row>
@@ -1093,11 +1093,11 @@
         <v>1226</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>885</v>
+        <v>937</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>72%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Food &amp; Beverage, Retail, Inventory &amp; Procurement</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, White Label &amp; CMS, Transport</t>
         </is>
       </c>
     </row>
@@ -1139,17 +1139,17 @@
         <v>1632</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1393</v>
+        <v>1548</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Seat Management &amp; Venue Maps, White Label &amp; CMS, Transport, Food &amp; Beverage, Retail, Inventory &amp; Procurement, Resources &amp; Capacity, Virtual Queue</t>
+          <t>Foundation &amp; Setup, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, White Label &amp; CMS, Marketing &amp; CRM, AI &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -1181,11 +1181,11 @@
         <v>1523</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1506</v>
+        <v>1523</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>99%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, White Label &amp; CMS, Food &amp; Beverage, Retail, Admission &amp; Access Control, Finance, Ledger &amp; Tax, Reporting &amp; Analytics, Marketing &amp; CRM, AI &amp; Intelligence</t>
+          <t>Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Transport, Food &amp; Beverage, Retail, Inventory &amp; Procurement, Admission &amp; Access Control, Accreditation, Resources &amp; Capacity, Workforce &amp; Staff, Maintenance &amp; Safety, Games &amp; Rides</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
         <v>1632</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1629</v>
+        <v>1632</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Subscription &amp; Licensing, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Transport, Food &amp; Beverage, Retail, Inventory &amp; Procurement, Accreditation, Resources &amp; Capacity, Workforce &amp; Staff, Maintenance &amp; Safety</t>
+          <t>Identity, Roles &amp; Security, Subscription &amp; Licensing, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Virtual Queue, Reporting &amp; Analytics, Marketing &amp; CRM, AI &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, AI &amp; Intelligence</t>
+          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Rentals, Admission &amp; Access Control, Accreditation, Workforce &amp; Staff, Finance, Ledger &amp; Tax, Reporting &amp; Analytics, Marketing &amp; CRM, AI &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Food &amp; Beverage, Rentals</t>
+          <t>Platform Operations, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Transport, Food &amp; Beverage, Retail, Rentals, Inventory &amp; Procurement</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Transport, Food &amp; Beverage, Retail, Rentals, Inventory &amp; Procurement, Admission &amp; Access Control, Accreditation, Resources &amp; Capacity, Finance, Ledger &amp; Tax, AI &amp; Intelligence</t>
+          <t>Accreditation, Resources &amp; Capacity, Workforce &amp; Staff, Maintenance &amp; Safety, Games &amp; Rides, Virtual Queue, Marketing &amp; CRM, AI &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -1515,17 +1515,17 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Tanmay Dukhande, Pallavi Sawant, Surendra, New full-stack developer 2, New full-stack developer 1, Pradnya Yeram, Sanket Keluskar</t>
+          <t>Pallavi Sawant, Hrushikant Patkar, Surendra, Tanmay Dukhande, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 1, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>5 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Chitrangi Mestry, Pranay Shinde, Deep Khanvilkar, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, New full-stack developer 1</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, New full-stack developer 1, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -1622,22 +1622,22 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>6 Oct 2026</t>
+          <t>8 Oct 2026</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>29 Mar 2027</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Chitrangi Mestry</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Chitrangi Mestry, Deep Khanvilkar, Pranay Shinde, New full-stack developer 1, Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar</t>
+          <t>Chitrangi Mestry, Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Tanmay Dukhande, Pallavi Sawant, New full-stack developer 1, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -1683,17 +1683,17 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>19 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Pallavi Sawant, Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar, Chitrangi Mestry, Pranay Shinde, New full-stack developer 1</t>
+          <t>Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Pradnya Yeram, Pallavi Sawant, New full-stack developer 1, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -1739,17 +1739,17 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Tanmay Dukhande, New full-stack developer 1, New full-stack developer 2, Chinmay Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Surendra, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -1790,22 +1790,22 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>15 Apr 2027</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Deep Khanvilkar, Tanmay Dukhande, Surendra, Chinmay Patkar, Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Deep Khanvilkar, New full-stack developer 2, Chinmay Patkar, Chitrangi Mestry, Sanket Keluskar, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Deep Khanvilkar, Tanmay Dukhande, Pallavi Sawant, Chitrangi Mestry</t>
+          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Pallavi Sawant, Hrushikant Patkar, Chinmay Patkar, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -2024,12 +2024,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>22 Jan 2027</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>1-6</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -2098,12 +2098,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Surendra, Tanmay Dukhande, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar</t>
+          <t>Hrushikant Patkar, Pallavi Sawant, Surendra, Tanmay Dukhande, Chitrangi Mestry, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>17 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, New full-stack developer 1, Hrushikant Patkar, Tanmay Dukhande, Pradnya Yeram, Deep Khanvilkar</t>
+          <t>New full-stack developer 2, New full-stack developer 1, Deep Khanvilkar, Tanmay Dukhande, Pradnya Yeram, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2280,22 +2280,22 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Hrushikant Patkar, Tanmay Dukhande, New full-stack developer 1, Chitrangi Mestry, Pallavi Sawant</t>
+          <t>Surendra, Deep Khanvilkar, Chitrangi Mestry, Hrushikant Patkar, Pallavi Sawant, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -2344,22 +2344,22 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>2 Mar 2027</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>New full-stack developer 2</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Pranay Shinde, Pallavi Sawant, Chitrangi Mestry, New full-stack developer 1, Tanmay Dukhande</t>
+          <t>New full-stack developer 2, Pradnya Yeram, Chitrangi Mestry, Sanket Keluskar, Chinmay Patkar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, New full-stack developer 2, New full-stack developer 1, Hrushikant Patkar, Deep Khanvilkar, Pallavi Sawant</t>
+          <t>New full-stack developer 1, Pallavi Sawant, Hrushikant Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>8 Jan 2027</t>
+          <t>30 Dec 2026</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Surendra, Tanmay Dukhande, New full-stack developer 2, Hrushikant Patkar, Chinmay Patkar, Deep Khanvilkar</t>
+          <t>Pallavi Sawant, Deep Khanvilkar, Pradnya Yeram, Hrushikant Patkar, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -2536,12 +2536,12 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pallavi Sawant, New full-stack developer 1, Pranay Shinde, Chitrangi Mestry, Deep Khanvilkar</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -2600,12 +2600,12 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>25 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pallavi Sawant, Chinmay Patkar, Deep Khanvilkar, Chitrangi Mestry, Pradnya Yeram</t>
+          <t>Tanmay Dukhande, Deep Khanvilkar, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -2659,12 +2659,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>13 Oct 2026</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>18 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Surendra, Deep Khanvilkar, New full-stack developer 2</t>
+          <t>Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -2728,12 +2728,12 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>25 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Chitrangi Mestry, Deep Khanvilkar, Pradnya Yeram, Chinmay Patkar, Sanket Keluskar</t>
+          <t>Pranay Shinde, Chitrangi Mestry, New full-stack developer 1, New full-stack developer 2, Tanmay Dukhande, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>18 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Chitrangi Mestry, Surendra, Tanmay Dukhande, Sanket Keluskar, Chinmay Patkar</t>
+          <t>Pranay Shinde, Sanket Keluskar, Pradnya Yeram, Chinmay Patkar, Tanmay Dukhande, Chitrangi Mestry</t>
         </is>
       </c>
     </row>
@@ -2856,22 +2856,22 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Sanket Keluskar, Chinmay Patkar, New full-stack developer 1, Pradnya Yeram, Hrushikant Patkar</t>
+          <t>Chinmay Patkar, Pallavi Sawant, Chitrangi Mestry, New full-stack developer 1, New full-stack developer 2, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -2915,17 +2915,17 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>5 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>7 Jan 2027</t>
+          <t>23 Dec 2026</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Tanmay Dukhande, Deep Khanvilkar, Chinmay Patkar, New full-stack developer 1, Sanket Keluskar</t>
+          <t>Chitrangi Mestry, Tanmay Dukhande, Deep Khanvilkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -2984,22 +2984,22 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Hrushikant Patkar, Sanket Keluskar, Chinmay Patkar, Pradnya Yeram, Pallavi Sawant</t>
+          <t>Hrushikant Patkar, New full-stack developer 1, Sanket Keluskar, Chinmay Patkar, Deep Khanvilkar, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -3043,27 +3043,27 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>6 Oct 2026</t>
+          <t>8 Oct 2026</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>5 Apr 2027</t>
+          <t>24 Mar 2027</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-9</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1, Chitrangi Mestry</t>
+          <t>Deep Khanvilkar, Pradnya Yeram, Hrushikant Patkar, Chitrangi Mestry, Sanket Keluskar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -3112,22 +3112,22 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>18 Mar 2027</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>1-9</t>
+          <t>1-8</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Chitrangi Mestry, Pradnya Yeram, Chinmay Patkar, New full-stack developer 2, Deep Khanvilkar</t>
+          <t>New full-stack developer 1, Pranay Shinde, Pradnya Yeram, Chinmay Patkar, Hrushikant Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -3171,27 +3171,27 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>3 Mar 2027</t>
+          <t>19 Feb 2027</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>29 Mar 2027</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>8-10</t>
+          <t>7-9</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Chitrangi Mestry</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Chitrangi Mestry, New full-stack developer 1, Chinmay Patkar, Deep Khanvilkar, Surendra</t>
+          <t>Chitrangi Mestry, Tanmay Dukhande, Pradnya Yeram, New full-stack developer 2, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>31 Mar 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -3250,12 +3250,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Pallavi Sawant, Chitrangi Mestry, Deep Khanvilkar, New full-stack developer 2</t>
+          <t>Pallavi Sawant, Hrushikant Patkar, New full-stack developer 1, Chinmay Patkar, Deep Khanvilkar, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>2 Apr 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -3314,12 +3314,12 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Chinmay Patkar, Hrushikant Patkar, New full-stack developer 2, Sanket Keluskar, Chitrangi Mestry</t>
+          <t>Hrushikant Patkar, Sanket Keluskar, Pradnya Yeram, New full-stack developer 2, Chinmay Patkar, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -3363,27 +3363,27 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>19 Jan 2027</t>
+          <t>12 Jan 2027</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>14 Apr 2027</t>
+          <t>30 Mar 2027</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>6-10</t>
+          <t>5-9</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Surendra, Pallavi Sawant, New full-stack developer 2, Pranay Shinde</t>
+          <t>Pranay Shinde, New full-stack developer 1, Chinmay Patkar, Pallavi Sawant, Sanket Keluskar, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3432,12 +3432,12 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>12 Apr 2027</t>
+          <t>31 Mar 2027</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-9</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pradnya Yeram, Chitrangi Mestry, New full-stack developer 2, Pranay Shinde, Pallavi Sawant</t>
+          <t>Hrushikant Patkar, Pallavi Sawant, Pradnya Yeram, Deep Khanvilkar, Sanket Keluskar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -3496,22 +3496,22 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>13 Apr 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-9</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>New full-stack developer 2</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar, Tanmay Dukhande, Hrushikant Patkar, Sanket Keluskar, Deep Khanvilkar</t>
+          <t>New full-stack developer 2, Chitrangi Mestry, Pradnya Yeram, Tanmay Dukhande, Sanket Keluskar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>12 Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Chitrangi Mestry, Sanket Keluskar, Pranay Shinde, Surendra, Hrushikant Patkar</t>
+          <t>Surendra, Pranay Shinde, Chinmay Patkar, Tanmay Dukhande, New full-stack developer 2, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>19 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Pranay Shinde, New full-stack developer 1, Sanket Keluskar, Deep Khanvilkar, Pradnya Yeram</t>
+          <t>Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1, Chinmay Patkar, Pranay Shinde, Chitrangi Mestry</t>
         </is>
       </c>
     </row>
@@ -3688,22 +3688,22 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>13 Apr 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-9</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, New full-stack developer 1, Chinmay Patkar, Pradnya Yeram, Pranay Shinde, Deep Khanvilkar</t>
+          <t>Pallavi Sawant, Chinmay Patkar, Tanmay Dukhande, Chitrangi Mestry, New full-stack developer 2, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3752,22 +3752,22 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>5 Apr 2027</t>
+          <t>26 Mar 2027</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>1-10</t>
+          <t>1-9</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar, Chitrangi Mestry</t>
+          <t>Chinmay Patkar, Surendra, Pradnya Yeram, Pallavi Sawant, Tanmay Dukhande, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -3826,12 +3826,12 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, New full-stack developer 1, New full-stack developer 2, Chinmay Patkar, Pradnya Yeram, Tanmay Dukhande</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, Deep Khanvilkar, New full-stack developer 2, Hrushikant Patkar, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3875,12 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>15 Apr 2027</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -3890,12 +3890,12 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Deep Khanvilkar, Tanmay Dukhande, Surendra, Chinmay Patkar, Chitrangi Mestry</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Deep Khanvilkar, New full-stack developer 2, Chinmay Patkar, Chitrangi Mestry</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Deep Khanvilkar, Tanmay Dukhande</t>
+          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Pallavi Sawant, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>28 Dec 2026</t>
+          <t>15 Dec 2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -4089,12 +4089,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>5 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>5 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>8 Oct 2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar, New full-stack developer 2, New full-stack developer 1, Pranay Shinde</t>
+          <t>Deep Khanvilkar, Tanmay Dukhande, Sanket Keluskar, Hrushikant Patkar, Pranay Shinde, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>17 Mar 2027</t>
+          <t>1 Mar 2027</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, New full-stack developer 1, Surendra, New full-stack developer 2</t>
+          <t>Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, New full-stack developer 2, Surendra</t>
         </is>
       </c>
     </row>
@@ -4212,12 +4212,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>14 Oct 2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5 Apr 2027</t>
+          <t>26 Mar 2027</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Deep Khanvilkar, Hrushikant Patkar, Sanket Keluskar, Pallavi Sawant</t>
+          <t>Pranay Shinde, Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar, Chinmay Patkar, New full-stack developer 1</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>8 Mar 2027</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, New full-stack developer 1, New full-stack developer 2</t>
+          <t>Pradnya Yeram, Chitrangi Mestry, Chinmay Patkar, Pallavi Sawant, New full-stack developer 2, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -4294,12 +4294,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>28 Oct 2026</t>
+          <t>13 Oct 2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>19 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Deep Khanvilkar, Pranay Shinde, Tanmay Dukhande, Sanket Keluskar, New full-stack developer 2</t>
+          <t>Hrushikant Patkar, Deep Khanvilkar, Pranay Shinde, Tanmay Dukhande, New full-stack developer 1, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4340,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>16 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, New full-stack developer 1</t>
+          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, New full-stack developer 1</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Deep Khanvilkar, Tanmay Dukhande, Sanket Keluskar</t>
+          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>30 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Surendra, Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram, Chinmay Patkar, Sanket Keluskar</t>
+          <t>Chinmay Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar, Chitrangi Mestry, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>21 Dec 2026</t>
+          <t>29 Oct 2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Tanmay Dukhande, Chinmay Patkar, Sanket Keluskar, Deep Khanvilkar</t>
+          <t>Deep Khanvilkar, Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, New full-stack developer 2, Chinmay Patkar, Pradnya Yeram, Surendra, Pallavi Sawant</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram, Surendra</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ44"/>
+  <dimension ref="A1:AH44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -4575,8 +4575,6 @@
     <col width="3.2" customWidth="1" min="32" max="32"/>
     <col width="3.2" customWidth="1" min="33" max="33"/>
     <col width="3.2" customWidth="1" min="34" max="34"/>
-    <col width="3.2" customWidth="1" min="35" max="35"/>
-    <col width="3.2" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4666,8 +4664,6 @@
       <c r="AF1" s="3" t="inlineStr"/>
       <c r="AG1" s="3" t="inlineStr"/>
       <c r="AH1" s="3" t="inlineStr"/>
-      <c r="AI1" s="3" t="inlineStr"/>
-      <c r="AJ1" s="3" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr"/>
@@ -4824,16 +4820,6 @@
           <t>26 Apr</t>
         </is>
       </c>
-      <c r="AI2" s="4" t="inlineStr">
-        <is>
-          <t>03 May</t>
-        </is>
-      </c>
-      <c r="AJ2" s="4" t="inlineStr">
-        <is>
-          <t>10 May</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -4843,7 +4829,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
@@ -4851,7 +4837,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="E3" s="7" t="n"/>
@@ -4861,10 +4847,10 @@
       <c r="I3" s="7" t="n"/>
       <c r="J3" s="7" t="n"/>
       <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
+      <c r="L3" s="8" t="n"/>
+      <c r="M3" s="8" t="n"/>
+      <c r="N3" s="8" t="n"/>
+      <c r="O3" s="8" t="n"/>
       <c r="P3" s="8" t="n"/>
       <c r="Q3" s="8" t="n"/>
       <c r="R3" s="8" t="n"/>
@@ -4876,16 +4862,14 @@
       <c r="X3" s="8" t="n"/>
       <c r="Y3" s="8" t="n"/>
       <c r="Z3" s="8" t="n"/>
-      <c r="AA3" s="8" t="n"/>
-      <c r="AB3" s="8" t="n"/>
-      <c r="AC3" s="8" t="n"/>
+      <c r="AA3" s="6" t="n"/>
+      <c r="AB3" s="6" t="n"/>
+      <c r="AC3" s="6" t="n"/>
       <c r="AD3" s="6" t="n"/>
       <c r="AE3" s="6" t="n"/>
       <c r="AF3" s="6" t="n"/>
       <c r="AG3" s="6" t="n"/>
       <c r="AH3" s="6" t="n"/>
-      <c r="AI3" s="6" t="n"/>
-      <c r="AJ3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4903,7 +4887,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>22 Jan 2027</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="E4" s="7" t="n"/>
@@ -4918,10 +4902,6 @@
       <c r="N4" s="7" t="n"/>
       <c r="O4" s="7" t="n"/>
       <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-      <c r="R4" s="7" t="n"/>
-      <c r="S4" s="7" t="n"/>
-      <c r="T4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4931,7 +4911,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -4939,7 +4919,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="E5" s="7" t="n"/>
@@ -4962,8 +4942,6 @@
       <c r="X5" s="8" t="n"/>
       <c r="Y5" s="8" t="n"/>
       <c r="Z5" s="8" t="n"/>
-      <c r="AA5" s="8" t="n"/>
-      <c r="AB5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4981,7 +4959,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>17 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="E6" s="7" t="n"/>
@@ -5004,8 +4982,6 @@
       <c r="X6" s="8" t="n"/>
       <c r="Y6" s="8" t="n"/>
       <c r="Z6" s="8" t="n"/>
-      <c r="AA6" s="8" t="n"/>
-      <c r="AB6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5023,7 +4999,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="F7" s="7" t="n"/>
@@ -5042,8 +5018,6 @@
       <c r="X7" s="8" t="n"/>
       <c r="Y7" s="8" t="n"/>
       <c r="Z7" s="8" t="n"/>
-      <c r="AA7" s="8" t="n"/>
-      <c r="AB7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5053,7 +5027,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -5061,14 +5035,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
       <c r="L8" s="8" t="n"/>
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n"/>
@@ -5084,9 +5056,6 @@
       <c r="X8" s="8" t="n"/>
       <c r="Y8" s="8" t="n"/>
       <c r="Z8" s="8" t="n"/>
-      <c r="AA8" s="8" t="n"/>
-      <c r="AB8" s="8" t="n"/>
-      <c r="AC8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5096,7 +5065,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>New full-stack developer 2</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -5104,7 +5073,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>2 Mar 2027</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -5125,9 +5094,6 @@
       <c r="X9" s="8" t="n"/>
       <c r="Y9" s="8" t="n"/>
       <c r="Z9" s="8" t="n"/>
-      <c r="AA9" s="8" t="n"/>
-      <c r="AB9" s="8" t="n"/>
-      <c r="AC9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5137,7 +5103,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5145,7 +5111,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>19 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -5164,8 +5130,6 @@
       <c r="X10" s="8" t="n"/>
       <c r="Y10" s="8" t="n"/>
       <c r="Z10" s="8" t="n"/>
-      <c r="AA10" s="8" t="n"/>
-      <c r="AB10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5175,7 +5139,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5183,7 +5147,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8 Jan 2027</t>
+          <t>30 Dec 2026</t>
         </is>
       </c>
       <c r="F11" s="7" t="n"/>
@@ -5192,13 +5156,9 @@
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
+      <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="8" t="n"/>
-      <c r="R11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -5216,7 +5176,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="E12" s="7" t="n"/>
@@ -5227,12 +5187,12 @@
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="8" t="n"/>
+      <c r="P12" s="8" t="n"/>
       <c r="Q12" s="8" t="n"/>
-      <c r="R12" s="7" t="n"/>
+      <c r="R12" s="8" t="n"/>
       <c r="S12" s="8" t="n"/>
       <c r="T12" s="8" t="n"/>
       <c r="U12" s="8" t="n"/>
@@ -5243,14 +5203,12 @@
       <c r="Z12" s="8" t="n"/>
       <c r="AA12" s="8" t="n"/>
       <c r="AB12" s="8" t="n"/>
-      <c r="AC12" s="8" t="n"/>
-      <c r="AD12" s="8" t="n"/>
+      <c r="AC12" s="6" t="n"/>
+      <c r="AD12" s="6" t="n"/>
       <c r="AE12" s="6" t="n"/>
       <c r="AF12" s="6" t="n"/>
       <c r="AG12" s="6" t="n"/>
       <c r="AH12" s="6" t="n"/>
-      <c r="AI12" s="6" t="n"/>
-      <c r="AJ12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5268,7 +5226,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
@@ -5279,9 +5237,6 @@
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
       <c r="P13" s="8" t="n"/>
       <c r="Q13" s="8" t="n"/>
       <c r="R13" s="8" t="n"/>
@@ -5293,9 +5248,6 @@
       <c r="X13" s="8" t="n"/>
       <c r="Y13" s="8" t="n"/>
       <c r="Z13" s="8" t="n"/>
-      <c r="AA13" s="8" t="n"/>
-      <c r="AB13" s="8" t="n"/>
-      <c r="AC13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5313,7 +5265,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>25 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="E14" s="7" t="n"/>
@@ -5324,6 +5276,7 @@
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
+      <c r="Q14" s="8" t="n"/>
       <c r="R14" s="8" t="n"/>
       <c r="S14" s="8" t="n"/>
       <c r="T14" s="8" t="n"/>
@@ -5334,8 +5287,6 @@
       <c r="Y14" s="8" t="n"/>
       <c r="Z14" s="8" t="n"/>
       <c r="AA14" s="8" t="n"/>
-      <c r="AB14" s="8" t="n"/>
-      <c r="AC14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5353,7 +5304,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="F15" s="7" t="n"/>
@@ -5363,10 +5314,8 @@
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
+      <c r="Q15" s="8" t="n"/>
+      <c r="R15" s="8" t="n"/>
       <c r="S15" s="8" t="n"/>
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="8" t="n"/>
@@ -5375,8 +5324,6 @@
       <c r="X15" s="8" t="n"/>
       <c r="Y15" s="8" t="n"/>
       <c r="Z15" s="8" t="n"/>
-      <c r="AA15" s="8" t="n"/>
-      <c r="AB15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5394,7 +5341,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>25 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="F16" s="7" t="n"/>
@@ -5403,12 +5350,7 @@
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="n"/>
+      <c r="Q16" s="8" t="n"/>
       <c r="R16" s="8" t="n"/>
       <c r="S16" s="8" t="n"/>
       <c r="T16" s="8" t="n"/>
@@ -5419,8 +5361,6 @@
       <c r="Y16" s="8" t="n"/>
       <c r="Z16" s="8" t="n"/>
       <c r="AA16" s="8" t="n"/>
-      <c r="AB16" s="8" t="n"/>
-      <c r="AC16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5438,7 +5378,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>18 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="F17" s="7" t="n"/>
@@ -5447,12 +5387,10 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
+      <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>
       <c r="Y17" s="8" t="n"/>
       <c r="Z17" s="8" t="n"/>
-      <c r="AA17" s="8" t="n"/>
-      <c r="AB17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5462,7 +5400,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -5470,7 +5408,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="E18" s="7" t="n"/>
@@ -5480,12 +5418,11 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
+      <c r="W18" s="8" t="n"/>
+      <c r="X18" s="8" t="n"/>
       <c r="Y18" s="8" t="n"/>
       <c r="Z18" s="8" t="n"/>
       <c r="AA18" s="8" t="n"/>
-      <c r="AB18" s="8" t="n"/>
-      <c r="AC18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5503,7 +5440,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>7 Jan 2027</t>
+          <t>23 Dec 2026</t>
         </is>
       </c>
       <c r="E19" s="7" t="n"/>
@@ -5513,13 +5450,8 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-      <c r="O19" s="7" t="n"/>
+      <c r="O19" s="8" t="n"/>
       <c r="P19" s="8" t="n"/>
-      <c r="Q19" s="8" t="n"/>
-      <c r="R19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5529,7 +5461,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -5537,7 +5469,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="E20" s="7" t="n"/>
@@ -5548,10 +5480,8 @@
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
+      <c r="R20" s="8" t="n"/>
+      <c r="S20" s="8" t="n"/>
       <c r="T20" s="8" t="n"/>
       <c r="U20" s="8" t="n"/>
       <c r="V20" s="8" t="n"/>
@@ -5561,8 +5491,6 @@
       <c r="Z20" s="8" t="n"/>
       <c r="AA20" s="8" t="n"/>
       <c r="AB20" s="8" t="n"/>
-      <c r="AC20" s="8" t="n"/>
-      <c r="AD20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -5572,7 +5500,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Chitrangi Mestry</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
@@ -5580,7 +5508,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>29 Mar 2027</t>
         </is>
       </c>
       <c r="E21" s="7" t="n"/>
@@ -5591,12 +5519,12 @@
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
+      <c r="Q21" s="6" t="n"/>
+      <c r="R21" s="8" t="n"/>
       <c r="S21" s="8" t="n"/>
       <c r="T21" s="8" t="n"/>
       <c r="U21" s="8" t="n"/>
@@ -5609,12 +5537,10 @@
       <c r="AB21" s="8" t="n"/>
       <c r="AC21" s="8" t="n"/>
       <c r="AD21" s="8" t="n"/>
-      <c r="AE21" s="9" t="n"/>
+      <c r="AE21" s="6" t="n"/>
       <c r="AF21" s="6" t="n"/>
       <c r="AG21" s="6" t="n"/>
       <c r="AH21" s="6" t="n"/>
-      <c r="AI21" s="6" t="n"/>
-      <c r="AJ21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5624,7 +5550,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -5632,7 +5558,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5 Apr 2027</t>
+          <t>24 Mar 2027</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -5643,10 +5569,7 @@
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
+      <c r="R22" s="8" t="n"/>
       <c r="S22" s="8" t="n"/>
       <c r="T22" s="8" t="n"/>
       <c r="U22" s="8" t="n"/>
@@ -5658,8 +5581,6 @@
       <c r="AA22" s="8" t="n"/>
       <c r="AB22" s="8" t="n"/>
       <c r="AC22" s="8" t="n"/>
-      <c r="AD22" s="8" t="n"/>
-      <c r="AE22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5669,7 +5590,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -5677,7 +5598,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1 Apr 2027</t>
+          <t>18 Mar 2027</t>
         </is>
       </c>
       <c r="G23" s="7" t="n"/>
@@ -5685,12 +5606,8 @@
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="7" t="n"/>
-      <c r="Q23" s="7" t="n"/>
+      <c r="R23" s="8" t="n"/>
+      <c r="S23" s="8" t="n"/>
       <c r="T23" s="8" t="n"/>
       <c r="U23" s="8" t="n"/>
       <c r="V23" s="8" t="n"/>
@@ -5700,8 +5617,6 @@
       <c r="Z23" s="8" t="n"/>
       <c r="AA23" s="8" t="n"/>
       <c r="AB23" s="8" t="n"/>
-      <c r="AC23" s="8" t="n"/>
-      <c r="AD23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5711,7 +5626,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pradnya Yeram</t>
+          <t>Chitrangi Mestry</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -5719,15 +5634,16 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
-        </is>
-      </c>
+          <t>29 Mar 2027</t>
+        </is>
+      </c>
+      <c r="X24" s="8" t="n"/>
+      <c r="Y24" s="8" t="n"/>
       <c r="Z24" s="8" t="n"/>
       <c r="AA24" s="8" t="n"/>
       <c r="AB24" s="8" t="n"/>
       <c r="AC24" s="8" t="n"/>
       <c r="AD24" s="8" t="n"/>
-      <c r="AE24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5737,7 +5653,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -5745,7 +5661,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>31 Mar 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="F25" s="7" t="n"/>
@@ -5753,11 +5669,8 @@
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
-      <c r="N25" s="7" t="n"/>
-      <c r="O25" s="7" t="n"/>
+      <c r="R25" s="8" t="n"/>
+      <c r="S25" s="8" t="n"/>
       <c r="T25" s="8" t="n"/>
       <c r="U25" s="8" t="n"/>
       <c r="V25" s="8" t="n"/>
@@ -5768,7 +5681,6 @@
       <c r="AA25" s="8" t="n"/>
       <c r="AB25" s="8" t="n"/>
       <c r="AC25" s="8" t="n"/>
-      <c r="AD25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -5778,7 +5690,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
@@ -5786,7 +5698,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>19 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="E26" s="6" t="n"/>
@@ -5797,12 +5709,12 @@
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="7" t="n"/>
       <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="n"/>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
-      <c r="Q26" s="7" t="n"/>
-      <c r="R26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6" t="n"/>
+      <c r="Q26" s="8" t="n"/>
+      <c r="R26" s="8" t="n"/>
       <c r="S26" s="8" t="n"/>
       <c r="T26" s="8" t="n"/>
       <c r="U26" s="8" t="n"/>
@@ -5816,11 +5728,9 @@
       <c r="AC26" s="8" t="n"/>
       <c r="AD26" s="8" t="n"/>
       <c r="AE26" s="9" t="n"/>
-      <c r="AF26" s="9" t="n"/>
-      <c r="AG26" s="9" t="n"/>
+      <c r="AF26" s="6" t="n"/>
+      <c r="AG26" s="6" t="n"/>
       <c r="AH26" s="6" t="n"/>
-      <c r="AI26" s="6" t="n"/>
-      <c r="AJ26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5830,7 +5740,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -5838,17 +5748,15 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2 Apr 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
+      <c r="Q27" s="8" t="n"/>
+      <c r="R27" s="8" t="n"/>
       <c r="S27" s="8" t="n"/>
       <c r="T27" s="8" t="n"/>
       <c r="U27" s="8" t="n"/>
@@ -5860,7 +5768,6 @@
       <c r="AA27" s="8" t="n"/>
       <c r="AB27" s="8" t="n"/>
       <c r="AC27" s="8" t="n"/>
-      <c r="AD27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5870,7 +5777,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -5878,9 +5785,10 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>14 Apr 2027</t>
-        </is>
-      </c>
+          <t>30 Mar 2027</t>
+        </is>
+      </c>
+      <c r="S28" s="8" t="n"/>
       <c r="T28" s="8" t="n"/>
       <c r="U28" s="8" t="n"/>
       <c r="V28" s="8" t="n"/>
@@ -5892,8 +5800,6 @@
       <c r="AB28" s="8" t="n"/>
       <c r="AC28" s="8" t="n"/>
       <c r="AD28" s="8" t="n"/>
-      <c r="AE28" s="9" t="n"/>
-      <c r="AF28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5911,7 +5817,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>12 Apr 2027</t>
+          <t>31 Mar 2027</t>
         </is>
       </c>
       <c r="F29" s="7" t="n"/>
@@ -5921,11 +5827,8 @@
       <c r="J29" s="7" t="n"/>
       <c r="K29" s="7" t="n"/>
       <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n"/>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="n"/>
-      <c r="Q29" s="7" t="n"/>
+      <c r="R29" s="8" t="n"/>
+      <c r="S29" s="8" t="n"/>
       <c r="T29" s="8" t="n"/>
       <c r="U29" s="8" t="n"/>
       <c r="V29" s="8" t="n"/>
@@ -5937,8 +5840,6 @@
       <c r="AB29" s="8" t="n"/>
       <c r="AC29" s="8" t="n"/>
       <c r="AD29" s="8" t="n"/>
-      <c r="AE29" s="9" t="n"/>
-      <c r="AF29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5948,7 +5849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>New full-stack developer 2</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -5956,11 +5857,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>13 Apr 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
+      <c r="S30" s="8" t="n"/>
       <c r="T30" s="8" t="n"/>
       <c r="U30" s="8" t="n"/>
       <c r="V30" s="8" t="n"/>
@@ -5972,8 +5873,6 @@
       <c r="AB30" s="8" t="n"/>
       <c r="AC30" s="8" t="n"/>
       <c r="AD30" s="8" t="n"/>
-      <c r="AE30" s="9" t="n"/>
-      <c r="AF30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5983,7 +5882,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -5991,16 +5890,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12 Apr 2027</t>
+          <t>5 Apr 2027</t>
         </is>
       </c>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
+      <c r="S31" s="8" t="n"/>
       <c r="T31" s="8" t="n"/>
       <c r="U31" s="8" t="n"/>
       <c r="V31" s="8" t="n"/>
@@ -6013,7 +5908,6 @@
       <c r="AC31" s="8" t="n"/>
       <c r="AD31" s="8" t="n"/>
       <c r="AE31" s="9" t="n"/>
-      <c r="AF31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6023,7 +5917,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -6031,15 +5925,15 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>19 Apr 2027</t>
+          <t>6 Apr 2027</t>
         </is>
       </c>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
+      <c r="S32" s="8" t="n"/>
+      <c r="T32" s="8" t="n"/>
       <c r="U32" s="8" t="n"/>
       <c r="V32" s="8" t="n"/>
       <c r="W32" s="8" t="n"/>
@@ -6051,8 +5945,6 @@
       <c r="AC32" s="8" t="n"/>
       <c r="AD32" s="8" t="n"/>
       <c r="AE32" s="9" t="n"/>
-      <c r="AF32" s="9" t="n"/>
-      <c r="AG32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6062,7 +5954,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -6070,7 +5962,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>13 Apr 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="F33" s="7" t="n"/>
@@ -6079,11 +5971,8 @@
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="n"/>
+      <c r="S33" s="8" t="n"/>
+      <c r="T33" s="8" t="n"/>
       <c r="U33" s="8" t="n"/>
       <c r="V33" s="8" t="n"/>
       <c r="W33" s="8" t="n"/>
@@ -6094,8 +5983,6 @@
       <c r="AB33" s="8" t="n"/>
       <c r="AC33" s="8" t="n"/>
       <c r="AD33" s="8" t="n"/>
-      <c r="AE33" s="9" t="n"/>
-      <c r="AF33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -6105,7 +5992,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
@@ -6113,7 +6000,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="E34" s="7" t="n"/>
@@ -6125,12 +6012,12 @@
       <c r="K34" s="7" t="n"/>
       <c r="L34" s="7" t="n"/>
       <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
-      <c r="O34" s="7" t="n"/>
-      <c r="P34" s="7" t="n"/>
-      <c r="Q34" s="7" t="n"/>
-      <c r="R34" s="7" t="n"/>
-      <c r="S34" s="7" t="n"/>
+      <c r="N34" s="6" t="n"/>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6" t="n"/>
+      <c r="Q34" s="6" t="n"/>
+      <c r="R34" s="8" t="n"/>
+      <c r="S34" s="8" t="n"/>
       <c r="T34" s="8" t="n"/>
       <c r="U34" s="8" t="n"/>
       <c r="V34" s="8" t="n"/>
@@ -6145,9 +6032,7 @@
       <c r="AE34" s="9" t="n"/>
       <c r="AF34" s="9" t="n"/>
       <c r="AG34" s="9" t="n"/>
-      <c r="AH34" s="9" t="n"/>
-      <c r="AI34" s="9" t="n"/>
-      <c r="AJ34" s="6" t="n"/>
+      <c r="AH34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6157,7 +6042,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -6165,7 +6050,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5 Apr 2027</t>
+          <t>26 Mar 2027</t>
         </is>
       </c>
       <c r="E35" s="7" t="n"/>
@@ -6175,8 +6060,7 @@
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
       <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
+      <c r="R35" s="8" t="n"/>
       <c r="S35" s="8" t="n"/>
       <c r="T35" s="8" t="n"/>
       <c r="U35" s="8" t="n"/>
@@ -6188,8 +6072,6 @@
       <c r="AA35" s="8" t="n"/>
       <c r="AB35" s="8" t="n"/>
       <c r="AC35" s="8" t="n"/>
-      <c r="AD35" s="8" t="n"/>
-      <c r="AE35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6199,7 +6081,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -6207,7 +6089,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="F36" s="7" t="n"/>
@@ -6218,12 +6100,7 @@
       <c r="K36" s="7" t="n"/>
       <c r="L36" s="7" t="n"/>
       <c r="M36" s="7" t="n"/>
-      <c r="N36" s="7" t="n"/>
-      <c r="O36" s="7" t="n"/>
-      <c r="P36" s="7" t="n"/>
-      <c r="Q36" s="7" t="n"/>
-      <c r="R36" s="7" t="n"/>
-      <c r="S36" s="7" t="n"/>
+      <c r="T36" s="8" t="n"/>
       <c r="U36" s="8" t="n"/>
       <c r="V36" s="8" t="n"/>
       <c r="W36" s="8" t="n"/>
@@ -6237,8 +6114,6 @@
       <c r="AE36" s="9" t="n"/>
       <c r="AF36" s="9" t="n"/>
       <c r="AG36" s="9" t="n"/>
-      <c r="AH36" s="9" t="n"/>
-      <c r="AI36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -6248,7 +6123,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
@@ -6256,7 +6131,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>15 Apr 2027</t>
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
@@ -6270,11 +6145,11 @@
       <c r="M37" s="7" t="n"/>
       <c r="N37" s="7" t="n"/>
       <c r="O37" s="7" t="n"/>
-      <c r="P37" s="7" t="n"/>
-      <c r="Q37" s="7" t="n"/>
-      <c r="R37" s="7" t="n"/>
-      <c r="S37" s="7" t="n"/>
-      <c r="T37" s="6" t="n"/>
+      <c r="P37" s="6" t="n"/>
+      <c r="Q37" s="6" t="n"/>
+      <c r="R37" s="6" t="n"/>
+      <c r="S37" s="8" t="n"/>
+      <c r="T37" s="8" t="n"/>
       <c r="U37" s="8" t="n"/>
       <c r="V37" s="8" t="n"/>
       <c r="W37" s="8" t="n"/>
@@ -6287,10 +6162,8 @@
       <c r="AD37" s="8" t="n"/>
       <c r="AE37" s="9" t="n"/>
       <c r="AF37" s="9" t="n"/>
-      <c r="AG37" s="9" t="n"/>
+      <c r="AG37" s="6" t="n"/>
       <c r="AH37" s="6" t="n"/>
-      <c r="AI37" s="6" t="n"/>
-      <c r="AJ37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6300,7 +6173,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -6308,7 +6181,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>15 Apr 2027</t>
         </is>
       </c>
       <c r="G38" s="7" t="n"/>
@@ -6320,10 +6193,8 @@
       <c r="M38" s="7" t="n"/>
       <c r="N38" s="7" t="n"/>
       <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
-      <c r="R38" s="7" t="n"/>
-      <c r="S38" s="7" t="n"/>
+      <c r="S38" s="8" t="n"/>
+      <c r="T38" s="8" t="n"/>
       <c r="U38" s="8" t="n"/>
       <c r="V38" s="8" t="n"/>
       <c r="W38" s="8" t="n"/>
@@ -6336,7 +6207,6 @@
       <c r="AD38" s="8" t="n"/>
       <c r="AE38" s="9" t="n"/>
       <c r="AF38" s="9" t="n"/>
-      <c r="AG38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -6354,7 +6224,7 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="E39" s="8" t="n"/>
@@ -6387,8 +6257,6 @@
       <c r="AF39" s="9" t="n"/>
       <c r="AG39" s="9" t="n"/>
       <c r="AH39" s="9" t="n"/>
-      <c r="AI39" s="9" t="n"/>
-      <c r="AJ39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6406,7 +6274,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="E40" s="8" t="n"/>
@@ -6439,8 +6307,6 @@
       <c r="AF40" s="9" t="n"/>
       <c r="AG40" s="9" t="n"/>
       <c r="AH40" s="9" t="n"/>
-      <c r="AI40" s="9" t="n"/>
-      <c r="AJ40" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6630,29 +6496,29 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18 Jan 2027</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>291</v>
+        <v>172</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>83</v>
+        <v>121</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>50</v>
+        <v>92</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>120</v>
@@ -6665,18 +6531,18 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>163</v>
+        <v>113</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>6.6</v>
+        <v>4.6</v>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Developer Portal &amp; Public API, Digital Asset Management, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
         </is>
       </c>
     </row>
@@ -6706,23 +6572,23 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>23 Dec 2026</t>
+          <t>18 Dec 2026</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>63</v>
+        <v>93</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J3" s="13" t="n">
         <v>98</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>112</v>
@@ -6741,18 +6607,18 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>6 May 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
-        <v>186</v>
+        <v>126</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>7.6</v>
+        <v>5.1</v>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Platform Operations, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Payments, Wallet &amp; Cashless</t>
+          <t>Foundation &amp; Setup, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Payments</t>
         </is>
       </c>
     </row>
@@ -6782,23 +6648,23 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>17 Dec 2026</t>
+          <t>16 Dec 2026</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>120</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>111</v>
+        <v>90</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>123</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>112</v>
@@ -6817,18 +6683,18 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>5 May 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>182</v>
+        <v>90</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>7.4</v>
+        <v>3.6</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
         </is>
       </c>
     </row>
@@ -6858,26 +6724,26 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>5 Jan 2027</t>
+          <t>8 Dec 2026</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>217</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>52</v>
+        <v>119</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>120</v>
@@ -6893,14 +6759,14 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>10 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>4.7</v>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
@@ -6969,18 +6835,18 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>28 Apr 2027</t>
+          <t>22 Apr 2027</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>5.6</v>
+        <v>4.3</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management</t>
         </is>
       </c>
     </row>
@@ -7010,29 +6876,29 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>21 Jan 2027</t>
+          <t>15 Dec 2026</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>317</v>
+        <v>112</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>120</v>
@@ -7045,18 +6911,18 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>5 May 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
-        <v>177</v>
+        <v>113</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>7.2</v>
+        <v>4.6</v>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps</t>
         </is>
       </c>
     </row>
@@ -7086,29 +6952,29 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>22 Jan 2027</t>
+          <t>15 Dec 2026</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>322</v>
+        <v>110</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>12</v>
+        <v>110</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>36</v>
+        <v>119</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>112</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>120</v>
@@ -7121,14 +6987,14 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>28 Apr 2027</t>
+          <t>15 Apr 2027</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>142</v>
+        <v>71</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>5.8</v>
+        <v>2.9</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
@@ -7197,18 +7063,18 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>26 Apr 2027</t>
+          <t>14 Apr 2027</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
-        <v>123</v>
+        <v>63</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps</t>
         </is>
       </c>
     </row>
@@ -7273,18 +7139,18 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>14 Apr 2027</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>4.3</v>
+        <v>2.3</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Digital Asset Management, Ticketing Catalogue &amp; Products</t>
         </is>
       </c>
     </row>
@@ -7321,10 +7187,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>38</v>
@@ -7349,18 +7215,18 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>30 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Subscription &amp; Licensing, Digital Asset Management, Ticketing Catalogue &amp; Products, Seat Management &amp; Venue Maps, Payments, Rentals</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Subscription &amp; Licensing, Ticketing Catalogue &amp; Products, Orders &amp; Reservations, Wallet &amp; Cashless, Admission &amp; Access Control, Resources &amp; Capacity</t>
         </is>
       </c>
     </row>
@@ -7421,18 +7287,18 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>3 May 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>161</v>
+        <v>91</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>9.1</v>
+        <v>5.2</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps</t>
+          <t>Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Wallet &amp; Cashless</t>
         </is>
       </c>
     </row>
@@ -7493,18 +7359,18 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>28 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
-        <v>143</v>
+        <v>91</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>8.1</v>
+        <v>5.2</v>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
+          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
         </is>
       </c>
     </row>
@@ -7534,11 +7400,11 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>23 Nov 2026</t>
+          <t>8 Dec 2026</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>121</v>
@@ -7610,11 +7476,11 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>23 Nov 2026</t>
+          <t>8 Dec 2026</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>121</v>

</xml_diff>

<commit_message>
TICVAI: Venue Management team builds the setup screens the Block A apps use first
Setup screens shared by Pallavi and Surendra (split by load and pace; Surendra had none and started
Venue Management waves 1-2 on day 1). Waves 1-2 only fill gaps: Block A work is placed first and never
moved by them. Pallavi's setup screens end 15 Oct, Surendra's 22 Oct; finish still 26 April.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Build Plan.xlsx
+++ b/ticvai/handoff/TICVAI - Build Plan.xlsx
@@ -1009,11 +1009,11 @@
         <v>1392</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1273</v>
+        <v>1281</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
         <v>1392</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1352</v>
+        <v>1346</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         <v>1226</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Hrushikant Patkar, Surendra, Tanmay Dukhande, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 1, Pradnya Yeram</t>
+          <t>Pallavi Sawant, Hrushikant Patkar, Tanmay Dukhande, Surendra, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 1, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, New full-stack developer 1, Pallavi Sawant</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, New full-stack developer 1, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>8 Oct 2026</t>
+          <t>7 Oct 2026</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Tanmay Dukhande, Pallavi Sawant, New full-stack developer 1, Sanket Keluskar</t>
+          <t>Chitrangi Mestry, Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Tanmay Dukhande, New full-stack developer 1, Pallavi Sawant, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>7 Oct 2026</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Pradnya Yeram, Pallavi Sawant, New full-stack developer 1, New full-stack developer 2</t>
+          <t>Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Pradnya Yeram, New full-stack developer 1, Pallavi Sawant, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>7 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Surendra, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, Surendra, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, Pradnya Yeram, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>14 Oct 2026</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -2034,12 +2034,12 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Surendra, Sanket Keluskar, Tanmay Dukhande, Pallavi Sawant, Pranay Shinde</t>
+          <t>Pallavi Sawant, Hrushikant Patkar, Sanket Keluskar, Tanmay Dukhande, Surendra, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pallavi Sawant, Surendra, Tanmay Dukhande, Chitrangi Mestry, Deep Khanvilkar</t>
+          <t>Hrushikant Patkar, Surendra, Pallavi Sawant, Tanmay Dukhande, Chitrangi Mestry, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>6 Oct 2026</t>
+          <t>5 Oct 2026</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Pallavi Sawant, Hrushikant Patkar, Deep Khanvilkar</t>
+          <t>New full-stack developer 1, Pallavi Sawant, Hrushikant Patkar, Deep Khanvilkar, Surendra</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Pallavi Sawant</t>
+          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>8 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Deep Khanvilkar, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, New full-stack developer 2</t>
+          <t>Tanmay Dukhande, Deep Khanvilkar, Chinmay Patkar, Pallavi Sawant, Sanket Keluskar, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>13 Oct 2026</t>
+          <t>9 Oct 2026</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>9 Oct 2026</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>15 Oct 2026</t>
+          <t>9 Oct 2026</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>8 Oct 2026</t>
+          <t>7 Oct 2026</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>15 Oct 2026</t>
+          <t>9 Oct 2026</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>12 Oct 2026</t>
+          <t>7 Oct 2026</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>14 Oct 2026</t>
+          <t>12 Oct 2026</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pallavi Sawant, Pradnya Yeram, Deep Khanvilkar, Sanket Keluskar, Pranay Shinde</t>
+          <t>Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Deep Khanvilkar, Sanket Keluskar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>15 Oct 2026</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>7 Oct 2026</t>
+          <t>6 Oct 2026</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -3762,12 +3762,12 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar, Surendra, Pradnya Yeram, Pallavi Sawant, Tanmay Dukhande, Sanket Keluskar</t>
+          <t>Surendra, Chinmay Patkar, Pradnya Yeram, Pallavi Sawant, Tanmay Dukhande, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>14 Oct 2026</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, New full-stack developer 2, Surendra</t>
+          <t>Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, Surendra, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Chitrangi Mestry, Chinmay Patkar, Pallavi Sawant, New full-stack developer 2, Sanket Keluskar</t>
+          <t>Pradnya Yeram, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar, New full-stack developer 2, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>16 Oct 2026</t>
+          <t>9 Oct 2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, New full-stack developer 1</t>
+          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, Surendra</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4417,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>13 Oct 2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar, Chitrangi Mestry, New full-stack developer 2</t>
+          <t>Chinmay Patkar, Pradnya Yeram, Sanket Keluskar, Pallavi Sawant, Chitrangi Mestry, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>26 Oct 2026</t>
+          <t>15 Oct 2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Chitrangi Mestry, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram, Surendra</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5307,6 +5307,7 @@
           <t>3 Mar 2027</t>
         </is>
       </c>
+      <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
@@ -5344,6 +5345,7 @@
           <t>12 Mar 2027</t>
         </is>
       </c>
+      <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
@@ -5381,6 +5383,7 @@
           <t>5 Mar 2027</t>
         </is>
       </c>
+      <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n"/>
@@ -5664,6 +5667,7 @@
           <t>22 Mar 2027</t>
         </is>
       </c>
+      <c r="E25" s="7" t="n"/>
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
@@ -5701,7 +5705,7 @@
           <t>6 Apr 2027</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
+      <c r="E26" s="7" t="n"/>
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n"/>
@@ -5751,6 +5755,7 @@
           <t>22 Mar 2027</t>
         </is>
       </c>
+      <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
@@ -6042,7 +6047,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>Surendra</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -6135,7 +6140,7 @@
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
+      <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
       <c r="H37" s="7" t="n"/>
       <c r="I37" s="7" t="n"/>
@@ -6184,6 +6189,7 @@
           <t>15 Apr 2027</t>
         </is>
       </c>
+      <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
@@ -6807,10 +6813,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="I6" s="2" t="n">
         <v>119</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>120</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>60</v>
@@ -7180,20 +7186,20 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>17 Nov 2026</t>
+          <t>16 Nov 2026</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>72</v>
@@ -7226,7 +7232,7 @@
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Subscription &amp; Licensing, Ticketing Catalogue &amp; Products, Orders &amp; Reservations, Wallet &amp; Cashless, Admission &amp; Access Control, Resources &amp; Capacity</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TICVAI: build plan rerun after r1 (finish 26 April holds; 13,590 h; ~1,290 overtime hours); deck v9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Build Plan.xlsx
+++ b/ticvai/handoff/TICVAI - Build Plan.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>16,238 points = 13,559 hours</t>
+          <t>16,275 points = 13,590 hours</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3,431 points = 2,865 hours</t>
+          <t>3,441 points = 2,873 hours</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>12,807 points = 10,694 hours</t>
+          <t>12,834 points = 10,716 hours</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>1,268 hours</t>
+          <t>1,293 hours</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1009,11 +1009,11 @@
         <v>1392</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1281</v>
+        <v>1260</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>92%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
         <v>1392</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1346</v>
+        <v>1353</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, White Label &amp; CMS, Transport, Food &amp; Beverage, Retail</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, White Label &amp; CMS, Transport, Food &amp; Beverage</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
         <v>1226</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>935</v>
+        <v>928</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, White Label &amp; CMS, Transport</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, White Label &amp; CMS, Transport, Food &amp; Beverage</t>
         </is>
       </c>
     </row>
@@ -1139,11 +1139,11 @@
         <v>1632</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1548</v>
+        <v>1573</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -1279,7 +1279,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Rentals, Admission &amp; Access Control, Accreditation, Workforce &amp; Staff, Finance, Ledger &amp; Tax, Reporting &amp; Analytics, Marketing &amp; CRM, AI &amp; Intelligence</t>
+          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Rentals, Admission &amp; Access Control, Accreditation, Workforce &amp; Staff, Finance, Ledger &amp; Tax, Marketing &amp; CRM, AI &amp; Intelligence</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Platform Operations, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Transport, Food &amp; Beverage, Retail, Rentals, Inventory &amp; Procurement</t>
+          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Payments, Wallet &amp; Cashless, Transport, Food &amp; Beverage, Retail</t>
         </is>
       </c>
     </row>
@@ -1494,19 +1494,19 @@
         <v>425</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3130</v>
+        <v>3150</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2613</v>
+        <v>2630</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1552</v>
+        <v>1563</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Hrushikant Patkar, Tanmay Dukhande, Surendra, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 1, Pradnya Yeram</t>
+          <t>Pallavi Sawant, Tanmay Dukhande, Hrushikant Patkar, New full-stack developer 1, Sanket Keluskar, Deep Khanvilkar, Surendra, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -1547,22 +1547,22 @@
         <v>866</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4363</v>
+        <v>4378</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>3641</v>
+        <v>3654</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2763</v>
+        <v>2769</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -1576,12 +1576,12 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, New full-stack developer 1, Pradnya Yeram</t>
+          <t>Chinmay Patkar, Pranay Shinde, Chitrangi Mestry, Tanmay Dukhande, Deep Khanvilkar, Pallavi Sawant, Pradnya Yeram, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry</t>
+          <t>Pradnya Yeram</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Tanmay Dukhande, New full-stack developer 1, Pallavi Sawant, Sanket Keluskar</t>
+          <t>Pradnya Yeram, Deep Khanvilkar, Chitrangi Mestry, Hrushikant Patkar, New full-stack developer 2, Sanket Keluskar, Tanmay Dukhande, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -1659,22 +1659,22 @@
         <v>411</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>507</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2356</v>
+        <v>2354</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1967</v>
+        <v>1965</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1777</v>
+        <v>1778</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -1683,17 +1683,17 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>8 Apr 2027</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Pradnya Yeram, New full-stack developer 1, Pallavi Sawant, New full-stack developer 2</t>
+          <t>Pallavi Sawant, Hrushikant Patkar, Pradnya Yeram, Chinmay Patkar, Tanmay Dukhande, New full-stack developer 2, Sanket Keluskar, Surendra</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Chitrangi Mestry, Surendra, Chinmay Patkar, Deep Khanvilkar, New full-stack developer 2, Pradnya Yeram, Hrushikant Patkar</t>
+          <t>New full-stack developer 1, Pradnya Yeram, Pallavi Sawant, Deep Khanvilkar, Tanmay Dukhande, Sanket Keluskar, Hrushikant Patkar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -1777,16 +1777,16 @@
         <v>264</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>177</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>15 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Deep Khanvilkar, New full-stack developer 2, Chinmay Patkar, Chitrangi Mestry, Sanket Keluskar, Pallavi Sawant</t>
+          <t>Pranay Shinde, Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1, Chitrangi Mestry, Surendra, Pradnya Yeram, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
         <v>114</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2748</v>
+        <v>2749</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Pallavi Sawant, Hrushikant Patkar, Chinmay Patkar, Pradnya Yeram</t>
+          <t>Kalpita Mejari, Second AI engineer, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Tanmay Dukhande, New full-stack developer 2, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -2009,13 +2009,13 @@
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -2076,10 +2076,10 @@
         <v>83</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -2098,12 +2098,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Surendra, Pallavi Sawant, Tanmay Dukhande, Chitrangi Mestry, Deep Khanvilkar</t>
+          <t>Deep Khanvilkar, Surendra, Tanmay Dukhande, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>3 Mar 2027</t>
+          <t>2 Mar 2027</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, New full-stack developer 1, Deep Khanvilkar, Tanmay Dukhande, Pradnya Yeram, Hrushikant Patkar</t>
+          <t>New full-stack developer 2, New full-stack developer 1, Hrushikant Patkar, Tanmay Dukhande, Pradnya Yeram, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2198,16 +2198,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>7</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Pradnya Yeram, Pranay Shinde, New full-stack developer 1, Tanmay Dukhande, Chitrangi Mestry</t>
+          <t>Pallavi Sawant, Tanmay Dukhande, New full-stack developer 1, Pradnya Yeram, Chitrangi Mestry</t>
         </is>
       </c>
     </row>
@@ -2268,10 +2268,10 @@
         <v>23</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -2290,12 +2290,12 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Surendra, Deep Khanvilkar, Chitrangi Mestry, Hrushikant Patkar, Pallavi Sawant, Pradnya Yeram</t>
+          <t>New full-stack developer 1, Hrushikant Patkar, Surendra, Tanmay Dukhande, Chitrangi Mestry, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2344,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -2354,12 +2354,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Pradnya Yeram, Chitrangi Mestry, Sanket Keluskar, Chinmay Patkar, Pranay Shinde</t>
+          <t>Deep Khanvilkar, Pradnya Yeram, Chitrangi Mestry, New full-stack developer 2, Chinmay Patkar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>3 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Pallavi Sawant, Hrushikant Patkar, Deep Khanvilkar, Surendra</t>
+          <t>Pallavi Sawant, Chinmay Patkar, New full-stack developer 1, Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Deep Khanvilkar, Pradnya Yeram, Hrushikant Patkar, Chinmay Patkar</t>
+          <t>New full-stack developer 1, Tanmay Dukhande, Sanket Keluskar, Hrushikant Patkar, Chinmay Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2509,25 +2509,25 @@
         <v>2</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>170</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>894</v>
+        <v>904</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>4 Mar 2027</t>
+          <t>15 Mar 2027</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -2546,12 +2546,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Deep Khanvilkar, Sanket Keluskar</t>
+          <t>Pranay Shinde, Tanmay Dukhande, Chinmay Patkar, Deep Khanvilkar, Chitrangi Mestry, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
         <v>533</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Deep Khanvilkar, Chinmay Patkar, Pallavi Sawant, Sanket Keluskar, New full-stack developer 2</t>
+          <t>Tanmay Dukhande, Chinmay Patkar, Pallavi Sawant, Sanket Keluskar, Chitrangi Mestry, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
         <v>272</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
@@ -2674,12 +2674,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Sanket Keluskar</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Sanket Keluskar, Deep Khanvilkar, New full-stack developer 2</t>
+          <t>Sanket Keluskar, New full-stack developer 2, Surendra, New full-stack developer 1, Deep Khanvilkar, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -2716,10 +2716,10 @@
         <v>211</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>12 Mar 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Chitrangi Mestry, New full-stack developer 1, New full-stack developer 2, Tanmay Dukhande, Chinmay Patkar</t>
+          <t>Pranay Shinde, Chitrangi Mestry, Chinmay Patkar, Tanmay Dukhande, Pradnya Yeram, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Sanket Keluskar, Pradnya Yeram, Chinmay Patkar, Tanmay Dukhande, Chitrangi Mestry</t>
+          <t>Pranay Shinde, Chitrangi Mestry, Pradnya Yeram, Chinmay Patkar, Surendra, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>12 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar, Pallavi Sawant, Chitrangi Mestry, New full-stack developer 1, New full-stack developer 2, Hrushikant Patkar</t>
+          <t>Pallavi Sawant, Chinmay Patkar, Surendra, New full-stack developer 2, New full-stack developer 1, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>23 Dec 2026</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Tanmay Dukhande, Deep Khanvilkar, Chinmay Patkar, Sanket Keluskar, Pranay Shinde</t>
+          <t>Chitrangi Mestry, Tanmay Dukhande, Chinmay Patkar, Deep Khanvilkar, Pradnya Yeram, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -2994,12 +2994,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, New full-stack developer 1, Sanket Keluskar, Chinmay Patkar, Deep Khanvilkar, Pradnya Yeram</t>
+          <t>Chinmay Patkar, Hrushikant Patkar, Sanket Keluskar, Chitrangi Mestry, Deep Khanvilkar, Pallavi Sawant</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>26 Mar 2027</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Pradnya Yeram</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Pradnya Yeram, Hrushikant Patkar, Chitrangi Mestry, Sanket Keluskar, Pranay Shinde</t>
+          <t>Pradnya Yeram, Hrushikant Patkar, Deep Khanvilkar, Chitrangi Mestry, Pallavi Sawant, Tanmay Dukhande</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3122,12 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Pranay Shinde, Pradnya Yeram, Chinmay Patkar, Hrushikant Patkar, Deep Khanvilkar</t>
+          <t>Chinmay Patkar, Tanmay Dukhande, Pradnya Yeram, Hrushikant Patkar, New full-stack developer 2, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Tanmay Dukhande, Pradnya Yeram, New full-stack developer 2, Hrushikant Patkar</t>
+          <t>Chitrangi Mestry, Deep Khanvilkar, Pradnya Yeram, New full-stack developer 2, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -3250,12 +3250,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Hrushikant Patkar, New full-stack developer 1, Chinmay Patkar, Deep Khanvilkar, Sanket Keluskar</t>
+          <t>Hrushikant Patkar, Sanket Keluskar, New full-stack developer 2, Pradnya Yeram, Deep Khanvilkar, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -3292,10 +3292,10 @@
         <v>101</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>23 Mar 2027</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Sanket Keluskar, Pradnya Yeram, New full-stack developer 2, Chinmay Patkar, Pallavi Sawant</t>
+          <t>Hrushikant Patkar, Pallavi Sawant, Sanket Keluskar, Pradnya Yeram, New full-stack developer 2, Chitrangi Mestry</t>
         </is>
       </c>
     </row>
@@ -3363,12 +3363,12 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>12 Jan 2027</t>
+          <t>8 Jan 2027</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>30 Mar 2027</t>
+          <t>31 Mar 2027</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -3378,12 +3378,12 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, New full-stack developer 1, Chinmay Patkar, Pallavi Sawant, Sanket Keluskar, Hrushikant Patkar</t>
+          <t>Chinmay Patkar, Hrushikant Patkar, Pallavi Sawant, Tanmay Dukhande, New full-stack developer 1, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>31 Mar 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -3442,12 +3442,12 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Pradnya Yeram, Pallavi Sawant, Deep Khanvilkar, Sanket Keluskar, Pranay Shinde</t>
+          <t>Pranay Shinde, Pradnya Yeram, Sanket Keluskar, Tanmay Dukhande, Surendra, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 2, Chitrangi Mestry, Pradnya Yeram, Tanmay Dukhande, Sanket Keluskar, Deep Khanvilkar</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, Chinmay Patkar, New full-stack developer 2, Deep Khanvilkar, Pranay Shinde</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>Surendra, Pranay Shinde, Chinmay Patkar, Tanmay Dukhande, New full-stack developer 2, Hrushikant Patkar</t>
+          <t>Surendra, Tanmay Dukhande, Pradnya Yeram, Deep Khanvilkar, Pranay Shinde, Hrushikant Patkar</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>8 Apr 2027</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1, Chinmay Patkar, Pranay Shinde, Chitrangi Mestry</t>
+          <t>Tanmay Dukhande, New full-stack developer 2, Pallavi Sawant, Chinmay Patkar, Hrushikant Patkar, Deep Khanvilkar</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>6</v>
@@ -3673,13 +3673,13 @@
         <v>11</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>47</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Pallavi Sawant, Chinmay Patkar, Tanmay Dukhande, Chitrangi Mestry, New full-stack developer 2, Hrushikant Patkar</t>
+          <t>Pallavi Sawant, Deep Khanvilkar, Chitrangi Mestry, Pranay Shinde, Hrushikant Patkar, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>26 Mar 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -3762,12 +3762,12 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Surendra, Chinmay Patkar, Pradnya Yeram, Pallavi Sawant, Tanmay Dukhande, Sanket Keluskar</t>
+          <t>New full-stack developer 1, Tanmay Dukhande, Pradnya Yeram, Sanket Keluskar, Pranay Shinde, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -3816,22 +3816,22 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>1-11</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Chitrangi Mestry, Deep Khanvilkar, New full-stack developer 2, Hrushikant Patkar, Pallavi Sawant</t>
+          <t>Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, Deep Khanvilkar, Hrushikant Patkar, Surendra</t>
         </is>
       </c>
     </row>
@@ -3868,10 +3868,10 @@
         <v>177</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>15 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -3890,12 +3890,12 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande, Pranay Shinde, Deep Khanvilkar, New full-stack developer 2, Chinmay Patkar, Chitrangi Mestry</t>
+          <t>Pranay Shinde, Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1, Chitrangi Mestry, Surendra</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
         <v>114</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>2748</v>
+        <v>2749</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>2863</v>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Sanket Keluskar, Pallavi Sawant, Hrushikant Patkar</t>
+          <t>Kalpita Mejari, Second AI engineer, Chinmay Patkar, Sanket Keluskar, Pranay Shinde, Tanmay Dukhande</t>
         </is>
       </c>
     </row>
@@ -4053,17 +4053,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>11 Dec 2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -4135,26 +4135,26 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
         <v>273</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>958</v>
+        <v>967</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Subscription &amp; Licensing, Identity, Roles &amp; Security, White Label &amp; CMS, Approval Workflows, Platform Operations, Tenancy, Venues &amp; Devices, Developer Portal &amp; Public API, Foundation &amp; Setup</t>
+          <t>Subscription &amp; Licensing, Identity, Roles &amp; Security, Platform Operations, White Label &amp; CMS, Approval Workflows, Tenancy, Venues &amp; Devices, Developer Portal &amp; Public API, Foundation &amp; Setup</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Tanmay Dukhande, Sanket Keluskar, Hrushikant Patkar, Pranay Shinde, Pallavi Sawant</t>
+          <t>Tanmay Dukhande, Deep Khanvilkar, Hrushikant Patkar, Sanket Keluskar, Pallavi Sawant, Surendra</t>
         </is>
       </c>
     </row>
@@ -4176,17 +4176,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1 Mar 2027</t>
+          <t>2 Mar 2027</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
         <v>158</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, Surendra, New full-stack developer 2</t>
+          <t>New full-stack developer 1, Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, New full-stack developer 2, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -4217,17 +4217,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>26 Mar 2027</t>
+          <t>23 Mar 2027</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1652</v>
+        <v>1660</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2162</v>
+        <v>2172</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -4236,7 +4236,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Pranay Shinde, Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar, Chinmay Patkar, New full-stack developer 1</t>
+          <t>Pranay Shinde, Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar, Sanket Keluskar, New full-stack developer 1</t>
         </is>
       </c>
     </row>
@@ -4258,17 +4258,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>8 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>1951</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Pradnya Yeram, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar, New full-stack developer 2, Sanket Keluskar</t>
+          <t>Pradnya Yeram, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar, New full-stack developer 2, Surendra</t>
         </is>
       </c>
     </row>
@@ -4299,26 +4299,26 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>8 Apr 2027</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>1165</v>
+        <v>1168</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Food &amp; Beverage, Foundation &amp; Setup, Inventory &amp; Procurement, Resources &amp; Capacity, Accreditation, Workforce &amp; Staff, Rentals, Maintenance &amp; Safety</t>
+          <t>Food &amp; Beverage, Foundation &amp; Setup, Inventory &amp; Procurement, Resources &amp; Capacity, Workforce &amp; Staff, Accreditation, Rentals, Maintenance &amp; Safety</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar, Deep Khanvilkar, Pranay Shinde, Tanmay Dukhande, New full-stack developer 1, New full-stack developer 2</t>
+          <t>Hrushikant Patkar, Deep Khanvilkar, Tanmay Dukhande, Pranay Shinde, New full-stack developer 1, Chinmay Patkar</t>
         </is>
       </c>
     </row>
@@ -4340,17 +4340,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>7 Apr 2027</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>1012</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1327</v>
+        <v>1324</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry, Pradnya Yeram, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, Surendra</t>
+          <t>Pradnya Yeram, Chitrangi Mestry, Pallavi Sawant, Chinmay Patkar, Sanket Keluskar, Surendra</t>
         </is>
       </c>
     </row>
@@ -4388,10 +4388,10 @@
         <v>177</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2881</v>
+        <v>2882</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>3058</v>
+        <v>3059</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Tanmay Dukhande, Hrushikant Patkar, Deep Khanvilkar</t>
+          <t>Kalpita Mejari, Second AI engineer, Pranay Shinde, Deep Khanvilkar, Hrushikant Patkar, Tanmay Dukhande</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>20 Apr 2027</t>
+          <t>16 Apr 2027</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Chinmay Patkar, Pradnya Yeram, Sanket Keluskar, Pallavi Sawant, Chitrangi Mestry, New full-stack developer 2</t>
+          <t>Sanket Keluskar, Chitrangi Mestry, Chinmay Patkar, New full-stack developer 1, New full-stack developer 2, Pradnya Yeram</t>
         </is>
       </c>
     </row>
@@ -4458,19 +4458,19 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>29 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
         <v>34</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>93</v>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar, Hrushikant Patkar, Chinmay Patkar, Sanket Keluskar</t>
+          <t>Deep Khanvilkar, Hrushikant Patkar, New full-stack developer 1, Chinmay Patkar, Sanket Keluskar</t>
         </is>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>New full-stack developer 1, Chitrangi Mestry, New full-stack developer 2, Pallavi Sawant, Pradnya Yeram, Sanket Keluskar</t>
+          <t>Pallavi Sawant, Pradnya Yeram, New full-stack developer 1, Surendra, Chitrangi Mestry, New full-stack developer 2</t>
         </is>
       </c>
     </row>
@@ -4833,11 +4833,11 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>2613</v>
+        <v>2630</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="E3" s="7" t="n"/>
@@ -4862,7 +4862,7 @@
       <c r="X3" s="8" t="n"/>
       <c r="Y3" s="8" t="n"/>
       <c r="Z3" s="8" t="n"/>
-      <c r="AA3" s="6" t="n"/>
+      <c r="AA3" s="8" t="n"/>
       <c r="AB3" s="6" t="n"/>
       <c r="AC3" s="6" t="n"/>
       <c r="AD3" s="6" t="n"/>
@@ -4883,7 +4883,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -4911,11 +4911,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3 Mar 2027</t>
+          <t>2 Mar 2027</t>
         </is>
       </c>
       <c r="E6" s="7" t="n"/>
@@ -4995,11 +4995,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>3 Mar 2027</t>
         </is>
       </c>
       <c r="F7" s="7" t="n"/>
@@ -5027,15 +5027,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5 Mar 2027</t>
+          <t>12 Mar 2027</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
@@ -5056,6 +5056,7 @@
       <c r="X8" s="8" t="n"/>
       <c r="Y8" s="8" t="n"/>
       <c r="Z8" s="8" t="n"/>
+      <c r="AA8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5065,7 +5066,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>Deep Khanvilkar</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -5073,7 +5074,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -5103,7 +5104,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5111,7 +5112,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3 Mar 2027</t>
+          <t>4 Mar 2027</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -5139,7 +5140,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5156,7 +5157,6 @@
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
-      <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="8" t="n"/>
     </row>
@@ -5168,11 +5168,11 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3641</v>
+        <v>3654</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -5218,15 +5218,15 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>894</v>
+        <v>904</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4 Mar 2027</t>
+          <t>15 Mar 2027</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
@@ -5237,6 +5237,7 @@
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
+      <c r="O13" s="8" t="n"/>
       <c r="P13" s="8" t="n"/>
       <c r="Q13" s="8" t="n"/>
       <c r="R13" s="8" t="n"/>
@@ -5248,6 +5249,8 @@
       <c r="X13" s="8" t="n"/>
       <c r="Y13" s="8" t="n"/>
       <c r="Z13" s="8" t="n"/>
+      <c r="AA13" s="8" t="n"/>
+      <c r="AB13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5261,7 +5264,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5296,11 +5299,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Sanket Keluskar</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5338,11 +5341,11 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>12 Mar 2027</t>
+          <t>16 Mar 2027</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
@@ -5363,6 +5366,7 @@
       <c r="Y16" s="8" t="n"/>
       <c r="Z16" s="8" t="n"/>
       <c r="AA16" s="8" t="n"/>
+      <c r="AB16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5403,7 +5407,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chinmay Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -5411,7 +5415,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>12 Mar 2027</t>
+          <t>5 Mar 2027</t>
         </is>
       </c>
       <c r="E18" s="7" t="n"/>
@@ -5425,7 +5429,6 @@
       <c r="X18" s="8" t="n"/>
       <c r="Y18" s="8" t="n"/>
       <c r="Z18" s="8" t="n"/>
-      <c r="AA18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5443,7 +5446,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>23 Dec 2026</t>
+          <t>25 Dec 2026</t>
         </is>
       </c>
       <c r="E19" s="7" t="n"/>
@@ -5464,7 +5467,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -5503,7 +5506,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Chitrangi Mestry</t>
+          <t>Pradnya Yeram</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
@@ -5522,7 +5525,7 @@
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
-      <c r="M21" s="6" t="n"/>
+      <c r="M21" s="7" t="n"/>
       <c r="N21" s="6" t="n"/>
       <c r="O21" s="6" t="n"/>
       <c r="P21" s="6" t="n"/>
@@ -5553,7 +5556,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Pradnya Yeram</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -5561,7 +5564,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>24 Mar 2027</t>
+          <t>26 Mar 2027</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -5593,7 +5596,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -5609,6 +5612,8 @@
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
       <c r="R23" s="8" t="n"/>
       <c r="S23" s="8" t="n"/>
       <c r="T23" s="8" t="n"/>
@@ -5656,7 +5661,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pallavi Sawant</t>
+          <t>Hrushikant Patkar</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -5672,7 +5677,6 @@
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="n"/>
       <c r="R25" s="8" t="n"/>
       <c r="S25" s="8" t="n"/>
       <c r="T25" s="8" t="n"/>
@@ -5694,15 +5698,15 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>1967</v>
+        <v>1965</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>8 Apr 2027</t>
         </is>
       </c>
       <c r="E26" s="7" t="n"/>
@@ -5748,11 +5752,11 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>22 Mar 2027</t>
+          <t>23 Mar 2027</t>
         </is>
       </c>
       <c r="E27" s="7" t="n"/>
@@ -5782,7 +5786,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pranay Shinde</t>
+          <t>Chinmay Patkar</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -5790,9 +5794,10 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>30 Mar 2027</t>
-        </is>
-      </c>
+          <t>31 Mar 2027</t>
+        </is>
+      </c>
+      <c r="R28" s="8" t="n"/>
       <c r="S28" s="8" t="n"/>
       <c r="T28" s="8" t="n"/>
       <c r="U28" s="8" t="n"/>
@@ -5814,7 +5819,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hrushikant Patkar</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -5822,7 +5827,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>31 Mar 2027</t>
+          <t>1 Apr 2027</t>
         </is>
       </c>
       <c r="F29" s="7" t="n"/>
@@ -5832,7 +5837,6 @@
       <c r="J29" s="7" t="n"/>
       <c r="K29" s="7" t="n"/>
       <c r="L29" s="7" t="n"/>
-      <c r="R29" s="8" t="n"/>
       <c r="S29" s="8" t="n"/>
       <c r="T29" s="8" t="n"/>
       <c r="U29" s="8" t="n"/>
@@ -5854,7 +5858,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New full-stack developer 2</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -5922,7 +5926,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Deep Khanvilkar</t>
+          <t>Tanmay Dukhande</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -5930,7 +5934,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6 Apr 2027</t>
+          <t>8 Apr 2027</t>
         </is>
       </c>
       <c r="F32" s="7" t="n"/>
@@ -5963,7 +5967,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -6005,7 +6009,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="E34" s="7" t="n"/>
@@ -6047,7 +6051,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Surendra</t>
+          <t>New full-stack developer 1</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -6055,16 +6059,13 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>26 Mar 2027</t>
+          <t>22 Mar 2027</t>
         </is>
       </c>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
       <c r="R35" s="8" t="n"/>
       <c r="S35" s="8" t="n"/>
       <c r="T35" s="8" t="n"/>
@@ -6086,7 +6087,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>New full-stack developer 1</t>
+          <t>Pallavi Sawant</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -6094,7 +6095,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="F36" s="7" t="n"/>
@@ -6128,15 +6129,15 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>15 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
@@ -6149,7 +6150,7 @@
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
       <c r="N37" s="7" t="n"/>
-      <c r="O37" s="7" t="n"/>
+      <c r="O37" s="6" t="n"/>
       <c r="P37" s="6" t="n"/>
       <c r="Q37" s="6" t="n"/>
       <c r="R37" s="6" t="n"/>
@@ -6167,7 +6168,7 @@
       <c r="AD37" s="8" t="n"/>
       <c r="AE37" s="9" t="n"/>
       <c r="AF37" s="9" t="n"/>
-      <c r="AG37" s="6" t="n"/>
+      <c r="AG37" s="9" t="n"/>
       <c r="AH37" s="6" t="n"/>
     </row>
     <row r="38">
@@ -6178,15 +6179,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tanmay Dukhande</t>
+          <t>Pranay Shinde</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="F38" s="7" t="n"/>
@@ -6198,7 +6199,6 @@
       <c r="L38" s="7" t="n"/>
       <c r="M38" s="7" t="n"/>
       <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
       <c r="S38" s="8" t="n"/>
       <c r="T38" s="8" t="n"/>
       <c r="U38" s="8" t="n"/>
@@ -6213,6 +6213,7 @@
       <c r="AD38" s="8" t="n"/>
       <c r="AE38" s="9" t="n"/>
       <c r="AF38" s="9" t="n"/>
+      <c r="AG38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -6498,7 +6499,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -6506,19 +6507,19 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>112</v>
@@ -6537,14 +6538,14 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
@@ -6574,27 +6575,27 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18 Dec 2026</t>
+          <t>21 Dec 2026</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="J3" s="13" t="n">
-        <v>98</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>118</v>
+        <v>120</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <v>123</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>112</v>
@@ -6613,18 +6614,18 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>26 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>5.1</v>
+        <v>3.7</v>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Payments</t>
+          <t>Foundation &amp; Setup, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Payments, Wallet &amp; Cashless</t>
         </is>
       </c>
     </row>
@@ -6650,7 +6651,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -6658,19 +6659,19 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>123</v>
+        <v>94</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>121</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>112</v>
@@ -6689,18 +6690,18 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>20 Apr 2027</t>
+          <t>26 Apr 2027</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>3.6</v>
+        <v>5.1</v>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Digital Asset Management, Ticketing Catalogue &amp; Products</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6727,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -6734,7 +6735,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>84</v>
@@ -6743,10 +6744,10 @@
         <v>117</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>112</v>
@@ -6765,14 +6766,14 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>23 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>4.7</v>
+        <v>4.1</v>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
@@ -6802,7 +6803,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -6813,13 +6814,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>119</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>120</v>
@@ -6841,18 +6842,18 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>22 Apr 2027</t>
+          <t>19 Apr 2027</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products</t>
         </is>
       </c>
     </row>
@@ -6878,27 +6879,27 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>15 Dec 2026</t>
+          <t>11 Dec 2026</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>112</v>
@@ -6921,14 +6922,14 @@
         </is>
       </c>
       <c r="R7" s="2" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="S7" s="2" t="n">
         <v>4.6</v>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps</t>
         </is>
       </c>
     </row>
@@ -6954,7 +6955,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -6962,19 +6963,19 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>110</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>119</v>
+        <v>107</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>123</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>112</v>
@@ -6993,18 +6994,18 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>15 Apr 2027</t>
+          <t>23 Apr 2027</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>2.9</v>
+        <v>4.7</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Digital Asset Management, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products</t>
         </is>
       </c>
     </row>
@@ -7030,7 +7031,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -7041,13 +7042,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>119</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>120</v>
@@ -7073,10 +7074,10 @@
         </is>
       </c>
       <c r="R9" s="2" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
@@ -7106,7 +7107,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -7117,7 +7118,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>94</v>
@@ -7145,18 +7146,18 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>14 Apr 2027</t>
+          <t>20 Apr 2027</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>2.3</v>
+        <v>3.6</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Digital Asset Management, Ticketing Catalogue &amp; Products</t>
+          <t>Foundation &amp; Setup, Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Approval Workflows, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7183,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -7193,10 +7194,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>36</v>
@@ -7225,7 +7226,7 @@
         </is>
       </c>
       <c r="R11" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="S11" s="2" t="n">
         <v>2.2</v>
@@ -7304,7 +7305,7 @@
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Developer Portal &amp; Public API, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Orders &amp; Reservations, Wallet &amp; Cashless</t>
+          <t>Tenancy, Venues &amp; Devices, Platform Operations, Subscription &amp; Licensing, Developer Portal &amp; Public API, Digital Asset Management, Ticketing Catalogue &amp; Products, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
         </is>
       </c>
     </row>
@@ -7365,18 +7366,18 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>20 Apr 2027</t>
+          <t>21 Apr 2027</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>Identity, Roles &amp; Security, Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations</t>
+          <t>Tenancy, Venues &amp; Devices, Subscription &amp; Licensing, Approval Workflows, Ticketing Catalogue &amp; Products, Pricing, Promotions &amp; Bundles, Seat Management &amp; Venue Maps, Orders &amp; Reservations, Wallet &amp; Cashless</t>
         </is>
       </c>
     </row>

</xml_diff>